<commit_message>
chore(excel): mở mẫu nhập ở sheet Hướng dẫn
</commit_message>
<xml_diff>
--- a/docs/ManagerDevice-Mau-Nhap-Thiet-Bi.xlsx
+++ b/docs/ManagerDevice-Mau-Nhap-Thiet-Bi.xlsx
@@ -4,17 +4,17 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Danh sách" state="hidden" r:id="rId4"/>
-    <sheet sheetId="2" name="Bộ lưu điện" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Laptop" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Màn hình" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Máy chiếu" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Máy in" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Máy scan" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Máy tính để bàn" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Thiết bị khác" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Thiết bị mạng" state="visible" r:id="rId13"/>
-    <sheet sheetId="11" name="Hướng dẫn" state="visible" r:id="rId14"/>
+    <sheet sheetId="11" name="Hướng dẫn" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Danh sách" state="hidden" r:id="rId5"/>
+    <sheet sheetId="2" name="Bộ lưu điện" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="Laptop" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="Màn hình" state="visible" r:id="rId8"/>
+    <sheet sheetId="5" name="Máy chiếu" state="visible" r:id="rId9"/>
+    <sheet sheetId="6" name="Máy in" state="visible" r:id="rId10"/>
+    <sheet sheetId="7" name="Máy scan" state="visible" r:id="rId11"/>
+    <sheet sheetId="8" name="Máy tính để bàn" state="visible" r:id="rId12"/>
+    <sheet sheetId="9" name="Thiết bị khác" state="visible" r:id="rId13"/>
+    <sheet sheetId="10" name="Thiết bị mạng" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="Ví dụ (không nhập)" state="hidden" r:id="rId15"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -1612,9 +1612,165 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="123">
   <si>
+    <t>HƯỚNG DẪN NHẬP THIẾT BỊ TỪ EXCEL</t>
+  </si>
+  <si>
+    <t>Mẫu này được tạo từ dữ liệu danh mục hiện có. Mỗi danh mục có một sheet riêng; chỉ nhập vào đúng sheet loại thiết bị.</t>
+  </si>
+  <si>
+    <t>QUY TẮC BẮT BUỘC</t>
+  </si>
+  <si>
+    <t>•  Mỗi dòng là một thiết bị. Không sửa tên cột, không chèn dòng phía trên dòng tiêu đề.</t>
+  </si>
+  <si>
+    <t>•  Tên thiết bị là bắt buộc, tối thiểu 2 ký tự.</t>
+  </si>
+  <si>
+    <t>•  Cột Danh mục có thể để trống — hệ thống tự dùng đúng danh mục của sheet đang nhập.</t>
+  </si>
+  <si>
+    <t>•  Trạng thái, Tình trạng, Bộ phận, Vị trí, Người sử dụng, Nhà cung cấp chỉ chọn từ dropdown để tránh sai dữ liệu.</t>
+  </si>
+  <si>
+    <t>•  Trạng thái "Đang sử dụng" bắt buộc phải chọn Người sử dụng. Nếu hệ thống chưa có nhân viên, trạng thái này sẽ không xuất hiện trong dropdown — hãy để trống hoặc chọn trạng thái khác.</t>
+  </si>
+  <si>
+    <t>•  Các cột thông số kỹ thuật (CPU, RAM, GPU, ổ cứng, hệ điều hành, tốc độ in…) có dropdown hoặc chỉ nhận số.</t>
+  </si>
+  <si>
+    <t>•  Ngày mua nhập dd/mm/yyyy. Tiền chỉ nhập số, không gõ "đ" hoặc dấu chấm phân cách.</t>
+  </si>
+  <si>
+    <t>•  Để trống Mã thiết bị nếu muốn hệ thống tự sinh mã theo danh mục.</t>
+  </si>
+  <si>
+    <t>•  Dòng trống được bỏ qua. Dòng lỗi sẽ được báo chi tiết, các dòng hợp lệ vẫn được nhập.</t>
+  </si>
+  <si>
+    <t>•  Các cột Bộ phận/Vị trí/Người sử dụng/Nhà cung cấp: để trống nếu chưa khai báo trong hệ thống, hoặc chọn đúng giá trị có sẵn.</t>
+  </si>
+  <si>
+    <t>DANH MỤC TRONG MẪU</t>
+  </si>
+  <si>
+    <t>Mã</t>
+  </si>
+  <si>
+    <t>Tên danh mục</t>
+  </si>
+  <si>
+    <t>Số trường thông số</t>
+  </si>
+  <si>
+    <t>UPS</t>
+  </si>
+  <si>
+    <t>Bộ lưu điện</t>
+  </si>
+  <si>
+    <t>LAPTOP</t>
+  </si>
+  <si>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>MONITOR</t>
+  </si>
+  <si>
+    <t>Màn hình</t>
+  </si>
+  <si>
+    <t>PROJECTOR</t>
+  </si>
+  <si>
+    <t>Máy chiếu</t>
+  </si>
+  <si>
+    <t>PRINTER</t>
+  </si>
+  <si>
+    <t>Máy in</t>
+  </si>
+  <si>
+    <t>SCANNER</t>
+  </si>
+  <si>
+    <t>Máy scan</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>Máy tính để bàn</t>
+  </si>
+  <si>
+    <t>OTHER</t>
+  </si>
+  <si>
+    <t>Thiết bị khác</t>
+  </si>
+  <si>
+    <t>NETWORK</t>
+  </si>
+  <si>
+    <t>Thiết bị mạng</t>
+  </si>
+  <si>
+    <t>VÍ DỤ CÁCH ĐIỀN</t>
+  </si>
+  <si>
     <t>Danh mục</t>
   </si>
   <si>
+    <t>Tên thiết bị / Cấu hình</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
+  </si>
+  <si>
+    <t>Máy tính để bàn Dell OptiPlex 7010</t>
+  </si>
+  <si>
+    <t>CPU: Intel Core i5-12400; RAM: 16 GB; Ổ cứng: SSD 512GB; OS: Windows 11 Pro</t>
+  </si>
+  <si>
+    <t>Laptop Dell Latitude 5440</t>
+  </si>
+  <si>
+    <t>CPU: Intel Core i7-1355U; RAM: 16 GB; Ổ cứng: SSD 1TB; OS: Windows 11 Pro</t>
+  </si>
+  <si>
+    <t>Máy in HP LaserJet Pro M404dn</t>
+  </si>
+  <si>
+    <t>Công nghệ in: Laser đen trắng; Khổ giấy: A4; Kết nối: USB + LAN</t>
+  </si>
+  <si>
+    <t>Máy scan Fujitsu fi-7160</t>
+  </si>
+  <si>
+    <t>Loại máy: ADF; Độ phân giải: 600 dpi; Khổ giấy: A4</t>
+  </si>
+  <si>
+    <t>QUY TRÌNH NHẬP</t>
+  </si>
+  <si>
+    <t>•  1. Mở đúng sheet danh mục (ví dụ "Máy in") và điền từng dòng thiết bị.</t>
+  </si>
+  <si>
+    <t>•  2. Lưu tệp dưới định dạng .xlsx.</t>
+  </si>
+  <si>
+    <t>•  3. Trong phần mềm: Thiết bị → Nhập Excel → chọn tệp vừa lưu.</t>
+  </si>
+  <si>
+    <t>•  4. Kiểm tra kết quả nhập; sửa các dòng báo lỗi rồi nhập lại nếu cần.</t>
+  </si>
+  <si>
+    <t>•  Nếu danh mục hoặc bộ phận/vị trí/nhân viên thay đổi, hãy tải lại mẫu mới từ phần mềm để cập nhật dropdown.</t>
+  </si>
+  <si>
     <t>Trạng thái</t>
   </si>
   <si>
@@ -1633,63 +1789,36 @@
     <t>Nhân viên</t>
   </si>
   <si>
-    <t>Bộ lưu điện</t>
-  </si>
-  <si>
     <t>Sẵn sàng</t>
   </si>
   <si>
     <t>Mới</t>
   </si>
   <si>
-    <t>Laptop</t>
-  </si>
-  <si>
     <t>Bảo trì</t>
   </si>
   <si>
     <t>Tốt</t>
   </si>
   <si>
-    <t>Màn hình</t>
-  </si>
-  <si>
     <t>Đã đặt trước</t>
   </si>
   <si>
     <t>Khá</t>
   </si>
   <si>
-    <t>Máy chiếu</t>
-  </si>
-  <si>
     <t>Đã thanh lý</t>
   </si>
   <si>
     <t>Kém</t>
   </si>
   <si>
-    <t>Máy in</t>
-  </si>
-  <si>
     <t>Thất lạc</t>
   </si>
   <si>
     <t>Hỏng</t>
   </si>
   <si>
-    <t>Máy scan</t>
-  </si>
-  <si>
-    <t>Máy tính để bàn</t>
-  </si>
-  <si>
-    <t>Thiết bị khác</t>
-  </si>
-  <si>
-    <t>Thiết bị mạng</t>
-  </si>
-  <si>
     <t>Mã thiết bị</t>
   </si>
   <si>
@@ -1729,9 +1858,6 @@
     <t>Số hóa đơn</t>
   </si>
   <si>
-    <t>Ghi chú</t>
-  </si>
-  <si>
     <t>Công suất</t>
   </si>
   <si>
@@ -1820,132 +1946,6 @@
   </si>
   <si>
     <t>Quản lý</t>
-  </si>
-  <si>
-    <t>HƯỚNG DẪN NHẬP THIẾT BỊ TỪ EXCEL</t>
-  </si>
-  <si>
-    <t>Mẫu này được tạo từ dữ liệu danh mục hiện có. Mỗi danh mục có một sheet riêng; chỉ nhập vào đúng sheet loại thiết bị.</t>
-  </si>
-  <si>
-    <t>QUY TẮC BẮT BUỘC</t>
-  </si>
-  <si>
-    <t>•  Mỗi dòng là một thiết bị. Không sửa tên cột, không chèn dòng phía trên dòng tiêu đề.</t>
-  </si>
-  <si>
-    <t>•  Tên thiết bị là bắt buộc, tối thiểu 2 ký tự.</t>
-  </si>
-  <si>
-    <t>•  Cột Danh mục có thể để trống — hệ thống tự dùng đúng danh mục của sheet đang nhập.</t>
-  </si>
-  <si>
-    <t>•  Trạng thái, Tình trạng, Bộ phận, Vị trí, Người sử dụng, Nhà cung cấp chỉ chọn từ dropdown để tránh sai dữ liệu.</t>
-  </si>
-  <si>
-    <t>•  Trạng thái "Đang sử dụng" bắt buộc phải chọn Người sử dụng. Nếu hệ thống chưa có nhân viên, trạng thái này sẽ không xuất hiện trong dropdown — hãy để trống hoặc chọn trạng thái khác.</t>
-  </si>
-  <si>
-    <t>•  Các cột thông số kỹ thuật (CPU, RAM, GPU, ổ cứng, hệ điều hành, tốc độ in…) có dropdown hoặc chỉ nhận số.</t>
-  </si>
-  <si>
-    <t>•  Ngày mua nhập dd/mm/yyyy. Tiền chỉ nhập số, không gõ "đ" hoặc dấu chấm phân cách.</t>
-  </si>
-  <si>
-    <t>•  Để trống Mã thiết bị nếu muốn hệ thống tự sinh mã theo danh mục.</t>
-  </si>
-  <si>
-    <t>•  Dòng trống được bỏ qua. Dòng lỗi sẽ được báo chi tiết, các dòng hợp lệ vẫn được nhập.</t>
-  </si>
-  <si>
-    <t>•  Các cột Bộ phận/Vị trí/Người sử dụng/Nhà cung cấp: để trống nếu chưa khai báo trong hệ thống, hoặc chọn đúng giá trị có sẵn.</t>
-  </si>
-  <si>
-    <t>DANH MỤC TRONG MẪU</t>
-  </si>
-  <si>
-    <t>Mã</t>
-  </si>
-  <si>
-    <t>Tên danh mục</t>
-  </si>
-  <si>
-    <t>Số trường thông số</t>
-  </si>
-  <si>
-    <t>UPS</t>
-  </si>
-  <si>
-    <t>LAPTOP</t>
-  </si>
-  <si>
-    <t>MONITOR</t>
-  </si>
-  <si>
-    <t>PROJECTOR</t>
-  </si>
-  <si>
-    <t>PRINTER</t>
-  </si>
-  <si>
-    <t>SCANNER</t>
-  </si>
-  <si>
-    <t>PC</t>
-  </si>
-  <si>
-    <t>OTHER</t>
-  </si>
-  <si>
-    <t>NETWORK</t>
-  </si>
-  <si>
-    <t>VÍ DỤ CÁCH ĐIỀN</t>
-  </si>
-  <si>
-    <t>Tên thiết bị / Cấu hình</t>
-  </si>
-  <si>
-    <t>Máy tính để bàn Dell OptiPlex 7010</t>
-  </si>
-  <si>
-    <t>CPU: Intel Core i5-12400; RAM: 16 GB; Ổ cứng: SSD 512GB; OS: Windows 11 Pro</t>
-  </si>
-  <si>
-    <t>Laptop Dell Latitude 5440</t>
-  </si>
-  <si>
-    <t>CPU: Intel Core i7-1355U; RAM: 16 GB; Ổ cứng: SSD 1TB; OS: Windows 11 Pro</t>
-  </si>
-  <si>
-    <t>Máy in HP LaserJet Pro M404dn</t>
-  </si>
-  <si>
-    <t>Công nghệ in: Laser đen trắng; Khổ giấy: A4; Kết nối: USB + LAN</t>
-  </si>
-  <si>
-    <t>Máy scan Fujitsu fi-7160</t>
-  </si>
-  <si>
-    <t>Loại máy: ADF; Độ phân giải: 600 dpi; Khổ giấy: A4</t>
-  </si>
-  <si>
-    <t>QUY TRÌNH NHẬP</t>
-  </si>
-  <si>
-    <t>•  1. Mở đúng sheet danh mục (ví dụ "Máy in") và điền từng dòng thiết bị.</t>
-  </si>
-  <si>
-    <t>•  2. Lưu tệp dưới định dạng .xlsx.</t>
-  </si>
-  <si>
-    <t>•  3. Trong phần mềm: Thiết bị → Nhập Excel → chọn tệp vừa lưu.</t>
-  </si>
-  <si>
-    <t>•  4. Kiểm tra kết quả nhập; sửa các dòng báo lỗi rồi nhập lại nếu cần.</t>
-  </si>
-  <si>
-    <t>•  Nếu danh mục hoặc bộ phận/vị trí/nhân viên thay đổi, hãy tải lại mẫu mới từ phần mềm để cập nhật dropdown.</t>
   </si>
   <si>
     <t>Tên thiết bị</t>
@@ -1995,14 +1995,6 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="1E3A8A"/>
       <sz val="15"/>
     </font>
@@ -2010,6 +2002,14 @@
       <b/>
       <color rgb="1E40AF"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFF"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2055,23 +2055,23 @@
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2419,101 +2419,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
+      <c r="A1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2540,83 +2540,83 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="23" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:23" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>69</v>
+      <c r="T1" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2672,121 +2672,121 @@
     <col min="3" max="3" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-    </row>
-    <row r="5" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
+      <c r="A7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
+      <c r="A8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
+      <c r="A9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
+      <c r="A10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
+      <c r="A12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
+      <c r="A13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
+      <c r="A14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-    </row>
-    <row r="17" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-    </row>
-    <row r="18" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>86</v>
+      <c r="A15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="17" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C19">
         <v>3</v>
@@ -2794,10 +2794,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C20">
         <v>9</v>
@@ -2805,10 +2805,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C21">
         <v>4</v>
@@ -2816,10 +2816,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C22">
         <v>4</v>
@@ -2827,10 +2827,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C23">
         <v>6</v>
@@ -2838,10 +2838,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C24">
         <v>5</v>
@@ -2849,10 +2849,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C25">
         <v>8</v>
@@ -2860,10 +2860,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -2871,118 +2871,118 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C27">
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-    </row>
-    <row r="30" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>39</v>
+    <row r="29" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+    </row>
+    <row r="30" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>99</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="C32" t="s">
-        <v>101</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B33" t="s">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="C33" t="s">
-        <v>103</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B34" t="s">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
+      <c r="A37" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
+      <c r="A38" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
+      <c r="A39" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
+      <c r="A40" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="B41" s="9"/>
-      <c r="C41" s="9"/>
+      <c r="A41" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -3018,44 +3018,44 @@
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>39</v>
+      <c r="C1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
         <v>113</v>
@@ -3067,10 +3067,10 @@
         <v>115</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="H2" t="s">
         <v>116</v>
@@ -3084,10 +3084,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
         <v>118</v>
@@ -3102,7 +3102,7 @@
         <v>121</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="H3" t="s">
         <v>122</v>
@@ -3138,80 +3138,80 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="22" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>42</v>
+      <c r="T1" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -3269,98 +3269,98 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="28" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:28" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>51</v>
+      <c r="T1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA1" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB1" s="8" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -3427,83 +3427,83 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="23" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:23" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>55</v>
+      <c r="T1" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -3564,83 +3564,83 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="23" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:23" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>58</v>
+      <c r="T1" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -3701,89 +3701,89 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="25" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:25" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:25" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>62</v>
+      <c r="T1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y1" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -3850,86 +3850,86 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="24" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:24" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:24" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>58</v>
+      <c r="T1" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -3996,95 +3996,95 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
     <col min="20" max="27" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:27" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:27" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>50</v>
+      <c r="T1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA1" s="8" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -4148,70 +4148,70 @@
     <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="6" customWidth="1"/>
     <col min="15" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R1" s="4" t="s">
+    <row r="1" ht="34" customHeight="1" spans="1:19" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(tools): bổ sung số nhân/luồng CPU, bus RAM, bộ nhớ GPU vào công cụ quét và danh mục
</commit_message>
<xml_diff>
--- a/docs/ManagerDevice-Mau-Nhap-Thiet-Bi.xlsx
+++ b/docs/ManagerDevice-Mau-Nhap-Thiet-Bi.xlsx
@@ -505,53 +505,81 @@
     <comment ref="U1" authorId="0">
       <text>
         <r>
+          <t>Chỉ nhập số (nhân).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0">
+      <text>
+        <r>
+          <t>Chỉ nhập số (luồng).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0">
+      <text>
+        <r>
           <t>Chỉ nhập số (GB).</t>
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0">
+    <comment ref="X1" authorId="0">
       <text>
         <r>
           <t>Chọn một giá trị: DDR4, DDR5, LPDDR4X, LPDDR5, LPDDR5X.</t>
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0">
+    <comment ref="Y1" authorId="0">
+      <text>
+        <r>
+          <t>Chỉ nhập số (MHz).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0">
       <text>
         <r>
           <t>Ví dụ: SSD 1TB.</t>
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0">
+    <comment ref="AA1" authorId="0">
       <text>
         <r>
           <t>Ví dụ: Intel Iris Xe.</t>
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0">
+    <comment ref="AB1" authorId="0">
+      <text>
+        <r>
+          <t>Ví dụ: 4GB hoặc Chia sẻ.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0">
       <text>
         <r>
           <t>Nhập giá trị thông số.</t>
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0">
+    <comment ref="AD1" authorId="0">
       <text>
         <r>
           <t>Chọn một giá trị: Windows 11 Pro, Windows 11 Home, Windows 10 Pro, Windows 10 Home, macOS, Ubuntu, Khác.</t>
         </r>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0">
+    <comment ref="AE1" authorId="0">
       <text>
         <r>
           <t>Chọn một giá trị: Có bản quyền, Không, Không rõ.</t>
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0">
+    <comment ref="AF1" authorId="0">
       <text>
         <r>
           <t>Chỉ nhập số (kg).</t>
@@ -1416,46 +1444,74 @@
     <comment ref="U1" authorId="0">
       <text>
         <r>
+          <t>Chỉ nhập số (nhân).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0">
+      <text>
+        <r>
+          <t>Chỉ nhập số (luồng).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0">
+      <text>
+        <r>
           <t>Chỉ nhập số (GB).</t>
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0">
+    <comment ref="X1" authorId="0">
       <text>
         <r>
           <t>Chọn một giá trị: DDR3, DDR4, DDR5.</t>
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0">
+    <comment ref="Y1" authorId="0">
+      <text>
+        <r>
+          <t>Chỉ nhập số (MHz).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0">
       <text>
         <r>
           <t>Ví dụ: SSD 512GB.</t>
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0">
+    <comment ref="AA1" authorId="0">
       <text>
         <r>
           <t>Ví dụ: Intel UHD 730.</t>
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0">
+    <comment ref="AB1" authorId="0">
+      <text>
+        <r>
+          <t>Ví dụ: 4GB hoặc Chia sẻ.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0">
       <text>
         <r>
           <t>Nhập giá trị thông số.</t>
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0">
+    <comment ref="AD1" authorId="0">
       <text>
         <r>
           <t>Chọn một giá trị: Windows 11 Pro, Windows 11 Home, Windows 10 Pro, Windows 10 Home, Ubuntu, Khác.</t>
         </r>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0">
+    <comment ref="AE1" authorId="0">
       <text>
         <r>
           <t>Chọn một giá trị: Có bản quyền, Không, Không rõ.</t>
@@ -1610,7 +1666,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="127">
   <si>
     <t>HƯỚNG DẪN NHẬP THIẾT BỊ TỪ EXCEL</t>
   </si>
@@ -1870,16 +1926,28 @@
     <t>CPU</t>
   </si>
   <si>
+    <t>Số nhân CPU (nhân)</t>
+  </si>
+  <si>
+    <t>Số luồng CPU (luồng)</t>
+  </si>
+  <si>
     <t>RAM (GB)</t>
   </si>
   <si>
     <t>Loại RAM</t>
   </si>
   <si>
+    <t>Bus RAM (MHz)</t>
+  </si>
+  <si>
     <t>Dung lượng ổ cứng</t>
   </si>
   <si>
     <t>Card đồ họa (GPU)</t>
+  </si>
+  <si>
+    <t>Bộ nhớ GPU</t>
   </si>
   <si>
     <t>Kích thước màn hình (inch)</t>
@@ -2607,16 +2675,16 @@
         <v>38</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="U1" s="8" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="W1" s="8" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2800,7 +2868,7 @@
         <v>20</v>
       </c>
       <c r="C20">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2855,7 +2923,7 @@
         <v>30</v>
       </c>
       <c r="C25">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3023,7 +3091,7 @@
         <v>36</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>72</v>
@@ -3058,13 +3126,13 @@
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F2" t="s">
         <v>59</v>
@@ -3073,13 +3141,13 @@
         <v>62</v>
       </c>
       <c r="H2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="I2">
         <v>18500000</v>
       </c>
       <c r="J2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -3090,28 +3158,28 @@
         <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G3" t="s">
         <v>62</v>
       </c>
       <c r="H3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I3">
         <v>6500000</v>
       </c>
       <c r="J3" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -3256,7 +3324,7 @@
   <sheetPr>
     <tabColor rgb="1E40AF"/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -3274,10 +3342,10 @@
     <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
-    <col min="20" max="28" width="22" customWidth="1"/>
+    <col min="20" max="32" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="34" customHeight="1" spans="1:32" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>69</v>
       </c>
@@ -3362,14 +3430,29 @@
       <c r="AB1" s="8" t="s">
         <v>93</v>
       </c>
+      <c r="AC1" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="AD1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="AE1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="AF1" s="8" t="s">
+        <v>97</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB1"/>
-  <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Bản quyền Windows trong danh sách có sẵn." sqref="AA2:AA500">
+  <autoFilter ref="A1:AF1"/>
+  <dataValidations count="15">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Hệ điều hành trong danh sách có sẵn." sqref="AD2:AD500">
+      <formula1>"Windows 11 Pro,Windows 11 Home,Windows 10 Pro,Windows 10 Home,macOS,Ubuntu,Khác"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Bản quyền Windows trong danh sách có sẵn." sqref="AE2:AE500">
       <formula1>"Có bản quyền,Không,Không rõ"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Khối lượng phải là số lớn hơn hoặc bằng 0." sqref="AB2:AB500">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Khối lượng phải là số lớn hơn hoặc bằng 0." sqref="AF2:AF500">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn danh mục trong danh sách có sẵn." sqref="C2:C500">
@@ -3393,14 +3476,20 @@
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Giá trị thanh lý phải là số lớn hơn hoặc bằng 0." sqref="Q2:Q500">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="RAM phải là số lớn hơn hoặc bằng 0." sqref="U2:U500">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Loại RAM trong danh sách có sẵn." sqref="V2:V500">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Số nhân CPU phải là số lớn hơn hoặc bằng 0." sqref="U2:U500">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Số luồng CPU phải là số lớn hơn hoặc bằng 0." sqref="V2:V500">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="RAM phải là số lớn hơn hoặc bằng 0." sqref="W2:W500">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Loại RAM trong danh sách có sẵn." sqref="X2:X500">
       <formula1>"DDR4,DDR5,LPDDR4X,LPDDR5,LPDDR5X"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Hệ điều hành trong danh sách có sẵn." sqref="Z2:Z500">
-      <formula1>"Windows 11 Pro,Windows 11 Home,Windows 10 Pro,Windows 10 Home,macOS,Ubuntu,Khác"</formula1>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Bus RAM phải là số lớn hơn hoặc bằng 0." sqref="Y2:Y500">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3494,16 +3583,16 @@
         <v>38</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="U1" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="W1" s="8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -3631,16 +3720,16 @@
         <v>38</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="U1" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="V1" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="V1" s="8" t="s">
-        <v>95</v>
-      </c>
       <c r="W1" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -3768,22 +3857,22 @@
         <v>38</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="U1" s="8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="W1" s="8" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="X1" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Y1" s="8" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -3917,19 +4006,19 @@
         <v>38</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="U1" s="8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="V1" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="W1" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="W1" s="8" t="s">
-        <v>103</v>
-      </c>
       <c r="X1" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -3983,7 +4072,7 @@
   <sheetPr>
     <tabColor rgb="1E40AF"/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -4001,10 +4090,10 @@
     <col min="17" max="17" width="16" style="6" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
-    <col min="20" max="27" width="22" customWidth="1"/>
+    <col min="20" max="31" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:27" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="34" customHeight="1" spans="1:31" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>69</v>
       </c>
@@ -4078,7 +4167,7 @@
         <v>89</v>
       </c>
       <c r="Y1" s="8" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="Z1" s="8" t="s">
         <v>91</v>
@@ -4086,11 +4175,26 @@
       <c r="AA1" s="8" t="s">
         <v>92</v>
       </c>
+      <c r="AB1" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="AE1" s="8" t="s">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA1"/>
-  <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Bản quyền Windows trong danh sách có sẵn." sqref="AA2:AA500">
+  <autoFilter ref="A1:AE1"/>
+  <dataValidations count="14">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Hệ điều hành trong danh sách có sẵn." sqref="AD2:AD500">
+      <formula1>"Windows 11 Pro,Windows 11 Home,Windows 10 Pro,Windows 10 Home,Ubuntu,Khác"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Bản quyền Windows trong danh sách có sẵn." sqref="AE2:AE500">
       <formula1>"Có bản quyền,Không,Không rõ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn danh mục trong danh sách có sẵn." sqref="C2:C500">
@@ -4114,14 +4218,20 @@
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Giá trị thanh lý phải là số lớn hơn hoặc bằng 0." sqref="Q2:Q500">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="RAM phải là số lớn hơn hoặc bằng 0." sqref="U2:U500">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Loại RAM trong danh sách có sẵn." sqref="V2:V500">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Số nhân CPU phải là số lớn hơn hoặc bằng 0." sqref="U2:U500">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Số luồng CPU phải là số lớn hơn hoặc bằng 0." sqref="V2:V500">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="RAM phải là số lớn hơn hoặc bằng 0." sqref="W2:W500">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Loại RAM trong danh sách có sẵn." sqref="X2:X500">
       <formula1>"DDR3,DDR4,DDR5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn Hệ điều hành trong danh sách có sẵn." sqref="Z2:Z500">
-      <formula1>"Windows 11 Pro,Windows 11 Home,Windows 10 Pro,Windows 10 Home,Ubuntu,Khác"</formula1>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Giá trị không hợp lệ" error="Bus RAM phải là số lớn hơn hoặc bằng 0." sqref="Y2:Y500">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(org): cơ cấu tổ chức theo Khối Đảng và Khối Nhà nước
- Thêm khối cơ quan cho phòng ban, nhân viên, thiết bị và báo cáo
- Cập nhật dữ liệu mẫu UBND xã An Bình, đồng bộ giao diện và Excel
- Chuẩn hóa thuật ngữ phòng ban, bỏ dependency không dùng
- Nâng phiên bản lên 1.0.2
</commit_message>
<xml_diff>
--- a/docs/ManagerDevice-Mau-Nhap-Thiet-Bi.xlsx
+++ b/docs/ManagerDevice-Mau-Nhap-Thiet-Bi.xlsx
@@ -1686,7 +1686,7 @@
     <t>•  Cột Danh mục có thể để trống — hệ thống tự dùng đúng danh mục của sheet đang nhập.</t>
   </si>
   <si>
-    <t>•  Trạng thái, Tình trạng, Bộ phận, Vị trí, Người sử dụng, Nhà cung cấp chỉ chọn từ dropdown để tránh sai dữ liệu.</t>
+    <t>•  Trạng thái, Tình trạng, Phòng ban, Vị trí, Người sử dụng, Nhà cung cấp chỉ chọn từ dropdown để tránh sai dữ liệu.</t>
   </si>
   <si>
     <t>•  Trạng thái "Đang sử dụng" bắt buộc phải chọn Người sử dụng. Nếu hệ thống chưa có nhân viên, trạng thái này sẽ không xuất hiện trong dropdown — hãy để trống hoặc chọn trạng thái khác.</t>
@@ -1704,7 +1704,7 @@
     <t>•  Dòng trống được bỏ qua. Dòng lỗi sẽ được báo chi tiết, các dòng hợp lệ vẫn được nhập.</t>
   </si>
   <si>
-    <t>•  Các cột Bộ phận/Vị trí/Người sử dụng/Nhà cung cấp: để trống nếu chưa khai báo trong hệ thống, hoặc chọn đúng giá trị có sẵn.</t>
+    <t>•  Các cột Phòng ban/Vị trí/Người sử dụng/Nhà cung cấp: để trống nếu chưa khai báo trong hệ thống, hoặc chọn đúng giá trị có sẵn.</t>
   </si>
   <si>
     <t>DANH MỤC TRONG MẪU</t>
@@ -1833,7 +1833,7 @@
     <t>Tình trạng</t>
   </si>
   <si>
-    <t>Bộ phận</t>
+    <t>Phòng ban</t>
   </si>
   <si>
     <t>Vị trí</t>

</xml_diff>